<commit_message>
updated burner annular design code
primary change was fixing the Aref formula.
</commit_message>
<xml_diff>
--- a/xjep_turbojet/station_data.xlsx
+++ b/xjep_turbojet/station_data.xlsx
@@ -580,25 +580,25 @@
         <v>0</v>
       </c>
       <c r="I3" t="n">
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
       <c r="J3" t="n">
-        <v>287.614</v>
+        <v>283.085</v>
       </c>
       <c r="K3" t="n">
-        <v>288.572</v>
+        <v>284.028</v>
       </c>
       <c r="L3" t="n">
-        <v>100.694</v>
+        <v>95.26000000000001</v>
       </c>
       <c r="M3" t="n">
-        <v>34.007</v>
+        <v>101.214</v>
       </c>
       <c r="N3" t="n">
-        <v>1.22</v>
+        <v>1.172</v>
       </c>
       <c r="O3" t="n">
-        <v>0.013</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="4">
@@ -627,25 +627,25 @@
         <v>0</v>
       </c>
       <c r="I4" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="J4" t="n">
-        <v>283.085</v>
+        <v>285.899</v>
       </c>
       <c r="K4" t="n">
-        <v>284.028</v>
+        <v>286.851</v>
       </c>
       <c r="L4" t="n">
-        <v>93.355</v>
+        <v>96.63800000000001</v>
       </c>
       <c r="M4" t="n">
-        <v>101.214</v>
+        <v>67.81</v>
       </c>
       <c r="N4" t="n">
-        <v>1.149</v>
+        <v>1.178</v>
       </c>
       <c r="O4" t="n">
-        <v>0.005</v>
+        <v>0.007</v>
       </c>
     </row>
     <row r="5">
@@ -700,43 +700,43 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>0.546</v>
+        <v>0.539</v>
       </c>
       <c r="C6" t="n">
-        <v>1510</v>
+        <v>1100</v>
       </c>
       <c r="D6" t="n">
         <v>377.617</v>
       </c>
       <c r="E6" t="n">
-        <v>1712.868</v>
+        <v>1184.076</v>
       </c>
       <c r="F6" t="n">
-        <v>0.336</v>
+        <v>0.283</v>
       </c>
       <c r="G6" t="n">
-        <v>0.016</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="H6" t="n">
-        <v>0.03</v>
+        <v>0.017</v>
       </c>
       <c r="I6" t="n">
         <v>0.4</v>
       </c>
       <c r="J6" t="n">
-        <v>1475.866</v>
+        <v>1072.807</v>
       </c>
       <c r="K6" t="n">
-        <v>1889.035</v>
+        <v>1279.891</v>
       </c>
       <c r="L6" t="n">
-        <v>341.015</v>
+        <v>340.306</v>
       </c>
       <c r="M6" t="n">
-        <v>295.601</v>
+        <v>254.722</v>
       </c>
       <c r="N6" t="n">
-        <v>0.805</v>
+        <v>1.105</v>
       </c>
       <c r="O6" t="n">
         <v>0.002</v>
@@ -747,43 +747,43 @@
         <v>5</v>
       </c>
       <c r="B7" t="n">
-        <v>0.546</v>
+        <v>0.539</v>
       </c>
       <c r="C7" t="n">
-        <v>1380.566</v>
+        <v>959.375</v>
       </c>
       <c r="D7" t="n">
-        <v>247.957</v>
+        <v>207.569</v>
       </c>
       <c r="E7" t="n">
-        <v>1549.964</v>
+        <v>1018.557</v>
       </c>
       <c r="F7" t="n">
-        <v>0.489</v>
+        <v>0.48</v>
       </c>
       <c r="G7" t="n">
-        <v>0.016</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="H7" t="n">
-        <v>0.031</v>
+        <v>0.018</v>
       </c>
       <c r="I7" t="n">
         <v>0.43</v>
       </c>
       <c r="J7" t="n">
-        <v>1344.101</v>
+        <v>931.237</v>
       </c>
       <c r="K7" t="n">
-        <v>1700.602</v>
+        <v>1085.182</v>
       </c>
       <c r="L7" t="n">
-        <v>220.361</v>
+        <v>183.941</v>
       </c>
       <c r="M7" t="n">
-        <v>303.765</v>
+        <v>256.086</v>
       </c>
       <c r="N7" t="n">
-        <v>0.571</v>
+        <v>0.6879999999999999</v>
       </c>
       <c r="O7" t="n">
         <v>0.003</v>
@@ -794,43 +794,43 @@
         <v>8</v>
       </c>
       <c r="B8" t="n">
-        <v>0.546</v>
+        <v>0.539</v>
       </c>
       <c r="C8" t="n">
-        <v>1380.566</v>
+        <v>959.375</v>
       </c>
       <c r="D8" t="n">
-        <v>247.957</v>
+        <v>207.569</v>
       </c>
       <c r="E8" t="n">
-        <v>1549.964</v>
+        <v>1018.557</v>
       </c>
       <c r="F8" t="n">
-        <v>0.489</v>
+        <v>0.48</v>
       </c>
       <c r="G8" t="n">
-        <v>0.016</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="H8" t="n">
-        <v>0.031</v>
+        <v>0.018</v>
       </c>
       <c r="I8" t="n">
         <v>1</v>
       </c>
       <c r="J8" t="n">
-        <v>1203.92</v>
+        <v>824.617</v>
       </c>
       <c r="K8" t="n">
-        <v>1523.24</v>
+        <v>960.936</v>
       </c>
       <c r="L8" t="n">
-        <v>135.611</v>
+        <v>112.279</v>
       </c>
       <c r="M8" t="n">
-        <v>668.579</v>
+        <v>560.42</v>
       </c>
       <c r="N8" t="n">
-        <v>0.392</v>
+        <v>0.474</v>
       </c>
       <c r="O8" t="n">
         <v>0.002</v>

</xml_diff>